<commit_message>
Schematic first draft, added datasheets, added partlist2 with some new components
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_1.xlsx
+++ b/schematic-design/Partslist_Group_PE04_1.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Projects\pe04\schematic-design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{464969A4-1B1D-407B-AA64-E37E3EC13834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{464969A4-1B1D-407B-AA64-E37E3EC13834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{898D3AE7-9E7D-4CFC-9175-944B93E1487F}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="52">
   <si>
     <t>Link</t>
   </si>
@@ -105,15 +105,6 @@
     <t>https://ee.hsrw.org/</t>
   </si>
   <si>
-    <t>Example Project</t>
-  </si>
-  <si>
-    <t>Stamm, Kremer</t>
-  </si>
-  <si>
-    <t>99</t>
-  </si>
-  <si>
     <t>Project</t>
   </si>
   <si>
@@ -175,6 +166,30 @@
   </si>
   <si>
     <t>https://www.mouser.de/ProductDetail/Analog-Devices/ADXL345BCCZ-RL7?qs=WIvQP4zGaninp9Gc%252BCsJzQ%3D%3D</t>
+  </si>
+  <si>
+    <t>81-PKM22EPPH4001-B0</t>
+  </si>
+  <si>
+    <t>PKM22EPPH4001-B0</t>
+  </si>
+  <si>
+    <t>Murata Electronics</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/Murata-Electronics/PKM22EPPH4001-B0?qs=flZjIlU0hx2Fke4m2iZ9MA%3D%3D</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>23/10/2025</t>
+  </si>
+  <si>
+    <t>Justin Chin Cheong, Abhinav Kothari</t>
+  </si>
+  <si>
+    <t>Knock Lock</t>
   </si>
 </sst>
 </file>
@@ -431,7 +446,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -517,41 +532,67 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -567,57 +608,27 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -637,6 +648,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -933,8 +948,8 @@
     <col min="2" max="2" width="4.88671875" customWidth="1"/>
     <col min="3" max="3" width="12.44140625" customWidth="1"/>
     <col min="4" max="4" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.77734375" customWidth="1"/>
-    <col min="6" max="6" width="7.77734375" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" customWidth="1"/>
     <col min="7" max="7" width="12.88671875" customWidth="1"/>
     <col min="8" max="8" width="8.6640625" customWidth="1"/>
     <col min="9" max="9" width="6.5546875" customWidth="1"/>
@@ -945,45 +960,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="43"/>
+      <c r="B1" s="44"/>
       <c r="C1" s="20" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="H1" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="21">
-        <v>43753</v>
+      <c r="B2" s="44"/>
+      <c r="C2" s="21" t="s">
+        <v>49</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
+      <c r="H2" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>6</v>
@@ -1018,19 +1033,19 @@
         <v>1</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" s="55" t="s">
         <v>38</v>
       </c>
+      <c r="E5" s="31" t="s">
+        <v>35</v>
+      </c>
       <c r="F5" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="56" t="s">
-        <v>39</v>
+        <v>30</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>36</v>
       </c>
       <c r="H5" s="24">
         <v>3.12</v>
@@ -1040,7 +1055,7 @@
         <v>3.12</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1051,19 +1066,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="33" t="s">
         <v>42</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" s="57" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" s="57" t="s">
-        <v>45</v>
       </c>
       <c r="H6" s="28">
         <v>5.65</v>
@@ -1072,26 +1087,42 @@
         <f t="shared" ref="I6:I19" si="0">B6*H6</f>
         <v>5.65</v>
       </c>
-      <c r="J6" s="58" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J6" s="34" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>3</v>
       </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="28"/>
+      <c r="B7" s="26">
+        <v>1</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="28">
+        <v>0.48199999999999998</v>
+      </c>
       <c r="I7" s="24">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J7" s="29"/>
+        <v>0.48199999999999998</v>
+      </c>
+      <c r="J7" s="34" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
@@ -1099,318 +1130,318 @@
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="27"/>
-      <c r="D8" s="26"/>
+      <c r="D8" s="27"/>
       <c r="E8" s="27"/>
       <c r="F8" s="27"/>
-      <c r="G8" s="26"/>
+      <c r="G8" s="27"/>
       <c r="H8" s="28"/>
       <c r="I8" s="24">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J8" s="29"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>5</v>
       </c>
-      <c r="B9" s="26"/>
+      <c r="B9" s="27"/>
       <c r="C9" s="27"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
       <c r="F9" s="27"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="24">
+      <c r="G9" s="27"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J9" s="29"/>
+      <c r="J9" s="34"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>6</v>
       </c>
-      <c r="B10" s="26"/>
+      <c r="B10" s="27"/>
       <c r="C10" s="27"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
       <c r="F10" s="27"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="24">
+      <c r="G10" s="27"/>
+      <c r="H10" s="52"/>
+      <c r="I10" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J10" s="29"/>
+      <c r="J10" s="34"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>7</v>
       </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="24">
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="54"/>
+      <c r="I11" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J11" s="33"/>
+      <c r="J11" s="55"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="9">
         <v>8</v>
       </c>
-      <c r="B12" s="30"/>
-      <c r="C12" s="31"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="24">
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="54"/>
+      <c r="I12" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J12" s="33"/>
+      <c r="J12" s="55"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="9">
         <v>9</v>
       </c>
-      <c r="B13" s="30"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="24">
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="54"/>
+      <c r="I13" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J13" s="33"/>
+      <c r="J13" s="55"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="9">
         <v>10</v>
       </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="24">
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J14" s="33"/>
+      <c r="J14" s="55"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="9">
         <v>11</v>
       </c>
-      <c r="B15" s="30"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="24">
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="54"/>
+      <c r="I15" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J15" s="33"/>
+      <c r="J15" s="55"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="9">
         <v>12</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="24">
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="54"/>
+      <c r="I16" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J16" s="33"/>
+      <c r="J16" s="55"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>13</v>
       </c>
-      <c r="B17" s="30"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="24">
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J17" s="33"/>
+      <c r="J17" s="55"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>14</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="24">
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="33"/>
+      <c r="J18" s="55"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="10">
         <v>15</v>
       </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="24">
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="56"/>
+      <c r="I19" s="53">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J19" s="37"/>
+      <c r="J19" s="57"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G20" s="40" t="s">
+      <c r="G20" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="H20" s="40"/>
+      <c r="H20" s="50"/>
       <c r="I20" s="13">
         <f>SUM(I5:I19)</f>
-        <v>8.77</v>
+        <v>9.2519999999999989</v>
       </c>
       <c r="J20" s="4"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="14" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
       <c r="E21" s="16"/>
-      <c r="G21" s="41" t="s">
+      <c r="G21" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="H21" s="41"/>
+      <c r="H21" s="51"/>
       <c r="I21" s="11">
         <f>I20*0.19</f>
-        <v>1.6662999999999999</v>
+        <v>1.7578799999999999</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="44" t="s">
+      <c r="A22" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="45"/>
+      <c r="B22" s="46"/>
       <c r="C22" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="45" t="s">
+      <c r="D22" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="48"/>
-      <c r="G22" s="41" t="s">
+      <c r="E22" s="47"/>
+      <c r="G22" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="H22" s="41"/>
+      <c r="H22" s="51"/>
       <c r="I22" s="12">
         <f>I20*1.19</f>
-        <v>10.436299999999999</v>
+        <v>11.009879999999999</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="46" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23" s="47"/>
+      <c r="A23" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="36"/>
       <c r="C23" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="40"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="51" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="52"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="46" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="47"/>
+      <c r="B24" s="36"/>
       <c r="C24" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="52"/>
+      <c r="E24" s="40"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="46" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25" s="47"/>
+      <c r="A25" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="36"/>
       <c r="C25" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="52"/>
+      <c r="E25" s="40"/>
       <c r="H25" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="49" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="50"/>
+      <c r="A26" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="38"/>
       <c r="C26" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="53" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="54"/>
+      <c r="E26" s="42"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="49" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="50"/>
+      <c r="A27" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="38"/>
       <c r="C27" s="19"/>
-      <c r="D27" s="53" t="s">
-        <v>36</v>
-      </c>
-      <c r="E27" s="54"/>
+      <c r="D27" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27" s="42"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
@@ -1510,6 +1541,16 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="D22:E22"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A27:B27"/>
@@ -1519,16 +1560,6 @@
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F19" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1540,9 +1571,11 @@
     <hyperlink ref="D24" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="D23" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="D26" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="J5" r:id="rId5" xr:uid="{98A04EE6-D62B-4687-AC62-05CBC3BC7F14}"/>
+    <hyperlink ref="J6" r:id="rId6" xr:uid="{9F9E23C2-0CE5-4F54-A453-2FB0482436B8}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId7"/>
   <headerFooter>
     <oddHeader>&amp;CParts list
 Practical Electronics</oddHeader>

</xml_diff>